<commit_message>
Publish the joining link for session 4
Prof. Mukul Aggarwal sent the link for Financial Intelligence and Fraud Analytics,
Monday 11:00-12:12. His name now carries his title, Prof., which he had not given
before. The session 4 chair sheet is regenerated with the link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/programme/chair-sheets/S04.xlsx
+++ b/programme/chair-sheets/S04.xlsx
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Session chair</t>
   </si>
   <si>
-    <t xml:space="preserve">Mukul Aggarwal</t>
+    <t xml:space="preserve">Prof. Mukul Aggarwal</t>
   </si>
   <si>
     <t xml:space="preserve">Co-chair</t>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">Joining link</t>
   </si>
   <si>
-    <t xml:space="preserve">to be confirmed</t>
+    <t xml:space="preserve">https://meet.google.com/jbq-wgwg-wbs</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>

</xml_diff>